<commit_message>
feat: add hero slider with dual salesforce trainers, batch updates, US contact, and brand styling
</commit_message>
<xml_diff>
--- a/backend/src/data/course_enrollments.xlsx
+++ b/backend/src/data/course_enrollments.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H9"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -565,9 +565,87 @@
         <v>Enrolled (Pending Fee Payment)</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>9/9/2026, 8:43:51 am IST</v>
+      </c>
+      <c r="B7" t="str">
+        <v>AA</v>
+      </c>
+      <c r="C7" t="str">
+        <v>aa@gmail.com</v>
+      </c>
+      <c r="D7" t="str">
+        <v>123456789</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Data Analytics with SQL, Power BI, Python, Excel</v>
+      </c>
+      <c r="F7" t="str">
+        <v>September 15, 2026 Batch | Weekday Batch (Mon to Fri) - 7:00 AM to 8:00 AM</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Job Seeker / Looking for Placement</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Enrolled (Pending Fee Payment)</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>9/9/2026, 8:47:18 am IST</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Abhi</v>
+      </c>
+      <c r="C8" t="str">
+        <v>abhi@gmail.com</v>
+      </c>
+      <c r="D8" t="str">
+        <v>9100449157</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Data Analytics with SQL, Power BI, Python, Excel</v>
+      </c>
+      <c r="F8" t="str">
+        <v>September 15, 2026 Batch | Weekend Batch (Sat &amp; Sun) - 6:00 PM to 8:00 PM IST</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Working Professional (IT)</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Enrolled (Pending Fee Payment)</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>9/9/2026, 8:53:33 am IST</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Praveen</v>
+      </c>
+      <c r="C9" t="str">
+        <v>praveen@gmail.com</v>
+      </c>
+      <c r="D9" t="str">
+        <v>9642384362</v>
+      </c>
+      <c r="E9" t="str">
+        <v>SQL for Data Analysts</v>
+      </c>
+      <c r="F9" t="str">
+        <v>September 15, 2026 | Weekend Batch (Sat &amp; Sun) - 6:00 PM to 8:00 PM IST</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Working Professional (IT)</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Enrolled (Pending Fee Payment)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add referral field to forms and elevate hero section with interactive bento studio
</commit_message>
<xml_diff>
--- a/backend/src/data/course_enrollments.xlsx
+++ b/backend/src/data/course_enrollments.xlsx
@@ -397,16 +397,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:K10"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
     <col min="3" max="3" width="28.83203125" customWidth="1"/>
     <col min="4" max="4" width="18.83203125" customWidth="1"/>
     <col min="5" max="5" width="45.83203125" customWidth="1"/>
-    <col min="6" max="6" width="30.83203125" customWidth="1"/>
-    <col min="7" max="7" width="25.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="45.83203125" customWidth="1"/>
     <col min="8" max="8" width="25.83203125" customWidth="1"/>
+    <col min="9" max="9" width="20.83203125" customWidth="1"/>
+    <col min="10" max="10" width="25.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -434,6 +436,15 @@
       <c r="H1" t="str">
         <v>Status</v>
       </c>
+      <c r="I1" t="str">
+        <v>Batch Start Date</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Batch Timings</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Referral</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -643,9 +654,41 @@
         <v>Enrolled (Pending Fee Payment)</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>9/9/2026, 9:56:34 pm IST</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Abhi</v>
+      </c>
+      <c r="C10" t="str">
+        <v>abhi@gmail.com</v>
+      </c>
+      <c r="D10" t="str">
+        <v>9100449157</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Data Analytics with SQL, Power BI, Python, Excel</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Working Professional (Non-IT / Switcher)</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Enrolled (Pending Fee Payment)</v>
+      </c>
+      <c r="I10" t="str">
+        <v>September 15, 2026 Batch</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Weekend Batch (Sat &amp; Sun) - 6:00 PM to 8:00 PM IST</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Mahesh</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>